<commit_message>
scan: seg5 2026-09-28 15:54 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq6_2026-09-24.xlsx
+++ b/output/full_scan/batch_seq6_2026-09-24.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>66.66258263654424</v>
+        <v>66.66258264529621</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>20.03638227562102</v>
+        <v>20.03638233254001</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>1.008072549259758</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.0279659061983181</v>
+        <v>0.0279659058479957</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>64.83174482953652</v>
+        <v>64.83174483637885</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>21.4997740037675</v>
+        <v>21.49977401398439</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>8.443961698534848</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>1.015667107052638</v>
+        <v>1.015667107145368</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>71.18692325866445</v>
+        <v>71.18692326537445</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>20.36263272905853</v>
+        <v>20.36263273942881</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2.24580486811646</v>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>63.0666188986628</v>
+        <v>63.06661889711793</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>14.68035603350259</v>
+        <v>14.68035599422468</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>1.897767706804681</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>1.320441410873102</v>
+        <v>1.320441410945215</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
         <v/>
       </c>
       <c r="D6" s="2" t="n">
-        <v>940.6269194686164</v>
+        <v>940.6269194686192</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>565</v>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>65.54270116081905</v>
+        <v>65.54270119928063</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>15.66891953482067</v>
+        <v>15.66891963656409</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>0.9584558643329044</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>4.653624494291645</v>
+        <v>4.653624493261205</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>68.11406770902241</v>
+        <v>68.11406773988737</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>43.05596085311367</v>
+        <v>43.05596087803512</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>1.350681376804406</v>
@@ -856,7 +856,7 @@
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>882.0855854405762</v>
+        <v>882.0855854405756</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1495</v>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>56.400107946741</v>
+        <v>56.40010796069737</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>19.34389631197316</v>
+        <v>19.34389638874685</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>1.349263704100556</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>12.90742260449349</v>
+        <v>12.90742260212381</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>58.26573932016866</v>
+        <v>58.26573933002864</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>15.61506634594098</v>
+        <v>15.61506640517012</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>1.74736065382166</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>1.446095108044223</v>
+        <v>1.446095107941201</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>856.3184997482543</v>
+        <v>856.3184997482542</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>132</v>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>63.59559106136845</v>
+        <v>63.59559110336602</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>22.17453390448567</v>
+        <v>22.17453390881341</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>1.069878972973927</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>2.69445116942654</v>
+        <v>2.69445116932351</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>57.91764608773407</v>
+        <v>57.91764609460841</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>24.12880708304367</v>
+        <v>24.12880710767694</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>0.3509783905401061</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-0.249979062613372</v>
+        <v>-0.2499790627163989</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>64.3875813106133</v>
+        <v>64.38758131685535</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>20.97541043626613</v>
+        <v>20.97541043588995</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.9196191487819916</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>3.835269044018928</v>
+        <v>3.835269043957112</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>56.07705364981348</v>
+        <v>56.07705361907149</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>28.24656522959186</v>
+        <v>28.24656523779491</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.409165748070089</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.4303852299350659</v>
+        <v>0.4303852295229902</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>43.5123613101049</v>
+        <v>43.51236130359737</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>30.01213485923392</v>
+        <v>30.0121348228333</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>10.36975850628528</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>-3.156081681665603</v>
+        <v>-3.156081681531665</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>62.65092002827535</v>
+        <v>62.65092003189135</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>30.71079744674877</v>
+        <v>30.71079743514897</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.2359423414332075</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.2252700331006494</v>
+        <v>0.2252700332861126</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>73.21134644791351</v>
+        <v>73.21134643791333</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>46.69088127013588</v>
+        <v>46.69088128627345</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.2929223485303</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>5.39644513611394</v>
+        <v>5.396445136484807</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>52.12986569519275</v>
+        <v>52.12986570728569</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>42.62926850747657</v>
+        <v>42.62926852689309</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.3708707727099934</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>-1.198090568126521</v>
+        <v>-1.198090568105901</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>62.63390265223265</v>
+        <v>62.63390267570716</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>23.28980005677465</v>
+        <v>23.28980001977224</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>2.259934107518183</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0.6575100139948079</v>
+        <v>0.6575100139226868</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>723.1294712635267</v>
+        <v>723.1294712635266</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>107.5</v>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>64.36927852414901</v>
+        <v>64.36927851827079</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>23.51868146081346</v>
+        <v>23.5186814405634</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>1.218678252716549</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>1.361157774871322</v>
+        <v>1.361157775118588</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>59.6111060781836</v>
+        <v>59.61110604525277</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>29.83339524561203</v>
+        <v>29.83339506359597</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.5071471822056217</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>-0.0336552233637077</v>
+        <v>-0.0336552234152223</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,7 +1559,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>56.17758028652718</v>
+        <v>56.17758027949982</v>
       </c>
       <c r="I21" s="2" t="n">
         <v>15.41856729698002</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>2.053150232184326</v>
+        <v>2.05315023241099</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>685.7153359639725</v>
+        <v>685.7153359639732</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>85.7</v>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>55.81718956452371</v>
+        <v>55.81718957299701</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>20.4142183625333</v>
+        <v>20.4142183801418</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.4982216913324923</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.4346386187129494</v>
+        <v>0.4346386188365926</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>63.79576574570996</v>
+        <v>63.79576576256471</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>18.39934887542577</v>
+        <v>18.39934889740825</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>1.430031148977345</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>1.789170172527805</v>
+        <v>1.789170172630829</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>683.9215222616863</v>
+        <v>683.9215222616861</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>157.5</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>62.08560633698952</v>
+        <v>62.08560634492002</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>18.47983130568164</v>
+        <v>18.47983131370662</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>2.269757034895909</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.6086841702846781</v>
+        <v>0.6086841704907591</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>63.50779681701987</v>
+        <v>63.50779682507245</v>
       </c>
       <c r="I25" s="2" t="n">
         <v>37.54616092363761</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-0.1797555502959937</v>
+        <v>-0.1797555503680925</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>64.06823281893976</v>
+        <v>64.06823286879842</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>30.43473403683808</v>
+        <v>30.43473402607072</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.5644020238586532</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>1.439548690416242</v>
+        <v>1.439548690457456</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>61.49437370620001</v>
+        <v>61.4943737089535</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>18.51541259867267</v>
+        <v>18.51541266220724</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.6017233650445784</v>
@@ -1916,7 +1916,7 @@
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>664.5775541717605</v>
+        <v>664.5775541717601</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>274</v>
@@ -1930,7 +1930,7 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>58.42997935578455</v>
+        <v>58.42997937481366</v>
       </c>
       <c r="I28" s="2" t="n">
         <v>28.20794361189195</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.5430680892161792</v>
+        <v>0.5430680888041124</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>53.58585285735273</v>
+        <v>53.5858527257891</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>27.55824196537597</v>
+        <v>27.5582420087473</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.3158218194710098</v>
@@ -2075,7 +2075,7 @@
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>640.72454781075</v>
+        <v>640.7245478107499</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>49.2</v>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>60.44000170734354</v>
+        <v>60.44000185171889</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>13.67839986329985</v>
+        <v>13.6783998427762</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.7238251276090925</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.2826127597924111</v>
+        <v>0.28261275960696</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>626.7572886142935</v>
+        <v>626.757288614293</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>320</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>57.56544904277526</v>
+        <v>57.56544905015739</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>14.23362223683571</v>
+        <v>14.23362223805619</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.5544628058873015</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>2.284717295549552</v>
+        <v>2.284717295858622</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>53.00848179598765</v>
+        <v>53.00848187069934</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>11.78606048173884</v>
+        <v>11.7860605299908</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.816426638421937</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.3757278517633402</v>
+        <v>0.3757278515469836</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>46.24721673166113</v>
+        <v>46.24721718938914</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>26.99637978708038</v>
+        <v>26.99637984701481</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.5352959447436444</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.0816399018393856</v>
+        <v>0.08163990101515189</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>54.12259619079699</v>
+        <v>54.12259641874993</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>11.19472339863702</v>
+        <v>11.1947234162119</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>1.106854266184539</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.2093845028315398</v>
+        <v>0.2093845028624441</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>56.29697327968442</v>
+        <v>56.29697321883355</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>20.87925687214075</v>
+        <v>20.87925688444003</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.8109296247975909</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.1093957968767523</v>
+        <v>0.1093957969159026</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>54.75179759228131</v>
+        <v>54.75179760268308</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>24.25431229264032</v>
+        <v>24.25431224395101</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.5113231867855531</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.2460884426102092</v>
+        <v>-0.2460884423938569</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2463,7 +2463,7 @@
         <v>51.94672572350459</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>4.579314553235909</v>
+        <v>4.579314586071396</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>2.038211037459534</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.2945727899367113</v>
+        <v>0.2945727899264081</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2499,7 +2499,7 @@
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>560.4207383764063</v>
+        <v>560.4207383764062</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>24.9</v>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>58.30571126287262</v>
+        <v>58.30571125283373</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>18.74010102092097</v>
+        <v>18.74010101154888</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.6981145641153743</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.0720673136884193</v>
+        <v>0.0720673137090254</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>54.98722876161556</v>
+        <v>54.98722877227682</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>9.775126547825019</v>
+        <v>9.775126560589136</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.4082512880279297</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>1.538349749933881</v>
+        <v>1.538349749727842</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2622,7 +2622,7 @@
         <v>62.34111175872214</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>10.72802222258614</v>
+        <v>10.7280222251487</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.6470188605997865</v>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>50.27569151227858</v>
+        <v>50.27569225450445</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>21.47895950619678</v>
+        <v>21.47895961386707</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.7738837136404555</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>1.263825371686212</v>
+        <v>1.263825345104759</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>52.79101167371908</v>
+        <v>52.79101168841078</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>8.098720366736252</v>
+        <v>8.098720347804557</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.8373601809609074</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>2.192723398495564</v>
+        <v>2.19272339866041</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>505.448080021483</v>
+        <v>505.4480800214831</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>24.9</v>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>49.58365134875887</v>
+        <v>49.58365129782495</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>8.538427455836214</v>
+        <v>8.538427430290829</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.6902568812034882</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.0105393242108474</v>
+        <v>0.0105393242520599</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>52.99368815352221</v>
+        <v>52.99368818698658</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>19.19277041623442</v>
+        <v>19.19277040414516</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>1.45478122683924</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>1.114227388121178</v>
+        <v>1.114227387709052</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>55.02064737640581</v>
+        <v>55.02064738750971</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>16.79100260769782</v>
+        <v>16.79100262295927</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.6755558163131483</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.1614099976816804</v>
+        <v>0.1614099976713774</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>51.76270051188474</v>
+        <v>51.76270038380225</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>29.62341744129527</v>
+        <v>29.62341746619241</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.1094152202160514</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.1191691632795219</v>
+        <v>-0.1191691628571076</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>49.27311121747557</v>
+        <v>49.27311124492324</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>20.97058091625856</v>
+        <v>20.97058091938624</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.5711946558878058</v>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>42.32645203887837</v>
+        <v>42.32645212393808</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>23.50530754835012</v>
+        <v>23.5053075816047</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.6067454909135692</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>1.321266692489797</v>
+        <v>1.321266691768631</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3082,7 +3082,7 @@
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>465.4414877189968</v>
+        <v>465.4414877189964</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>37.85</v>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>54.230999058813</v>
+        <v>54.23099885696675</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>20.29680733431054</v>
+        <v>20.29680774230329</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.9868653522617546</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.5286082147826853</v>
+        <v>0.5286082154111575</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,7 +3149,7 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>49.27003396441372</v>
+        <v>49.27003401400765</v>
       </c>
       <c r="I51" s="2" t="n">
         <v>20.17410291807317</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.4794189436569769</v>
+        <v>0.4794189435848568</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>46.34756951096985</v>
+        <v>46.34756962799259</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>11.48368397024404</v>
+        <v>11.48368400662731</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.9118758669782656</v>
@@ -3241,7 +3241,7 @@
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>459.9384265565117</v>
+        <v>459.9384265565353</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>30.55</v>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>65.91197423665392</v>
+        <v>65.9119741398849</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>18.56444067692023</v>
+        <v>18.56444068287822</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>1.673922534946038</v>
@@ -3308,7 +3308,7 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>50.72279301066639</v>
+        <v>50.72279302367088</v>
       </c>
       <c r="I54" s="2" t="n">
         <v>16.15653066207243</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.1864583540860164</v>
+        <v>0.1864583541066218</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>439.6646192834893</v>
+        <v>439.6646192834889</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>68.59999999999999</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>50.77775427177215</v>
+        <v>50.77775406772084</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>12.77166142359949</v>
+        <v>12.77166140010748</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.4768365100193492</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.1963630310635716</v>
+        <v>0.1963630318774921</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,7 +3414,7 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>44.71636053240834</v>
+        <v>44.7163605359483</v>
       </c>
       <c r="I56" s="2" t="n">
         <v>13.72835704790159</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-17.41231303223928</v>
+        <v>-17.41231303429979</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>50.69751580643432</v>
+        <v>50.69751589878662</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>14.93495377737909</v>
+        <v>14.93495370666925</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.3883922134014348</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.1803094864995612</v>
+        <v>0.1803094858813961</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>419.0415423013457</v>
+        <v>419.0415423013458</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>102</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>39.45290056819324</v>
+        <v>39.4529006043575</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>38.50243126639941</v>
+        <v>38.5024312396481</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>1.302163926499033</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.1976418202016896</v>
+        <v>0.1976418200574481</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>40.50182742669804</v>
+        <v>40.50182741793139</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>20.12072849354107</v>
+        <v>20.12072849093827</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.4322829297482632</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.4756110686105068</v>
+        <v>-0.4756110685796</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3612,7 +3612,7 @@
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>408.3472694522603</v>
+        <v>408.3472694522605</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>62</v>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>33.4157683350104</v>
+        <v>33.41576828373668</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>30.41685889535179</v>
+        <v>30.41685899161678</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.506398935503666</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.0502098099906191</v>
+        <v>0.050209810382142</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>404.2211869716203</v>
+        <v>404.2211869716205</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>37</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>62.30641641229285</v>
+        <v>62.30641638438206</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>16.87008102590127</v>
+        <v>16.87008103914424</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>7.103814350115726</v>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>38.3786495934306</v>
+        <v>38.37864969904653</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>35.19637842361337</v>
+        <v>35.19637843995342</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.4544712570610476</v>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>52.14845627375989</v>
+        <v>52.14845639667488</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>23.62827745762274</v>
+        <v>23.62827750772938</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.3275550635124111</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.1311472422851695</v>
+        <v>0.1311472423572883</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,7 +3838,7 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>49.36629717140195</v>
+        <v>49.3662971753635</v>
       </c>
       <c r="I64" s="2" t="n">
         <v>13.30479063962005</v>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>53.04440237537673</v>
+        <v>53.04440237315566</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>13.75830597246228</v>
+        <v>13.75830598057892</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.9214822437430756</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.2859364521955773</v>
+        <v>0.2859364522161847</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3947,7 +3947,7 @@
         <v>49.52662480919999</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>13.22340727407215</v>
+        <v>13.22340730764942</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.7822159383367108</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.3924543909837721</v>
+        <v>0.3924543911279985</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>51.65522475500319</v>
+        <v>51.65522489346169</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>14.35776240588586</v>
+        <v>14.35776235694837</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.3204236180844755</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.1226179573443029</v>
+        <v>0.1226179572618773</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4036,7 +4036,7 @@
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>374.887673000443</v>
+        <v>374.8876730004434</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>23.7</v>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>51.02435900770365</v>
+        <v>51.02435907135261</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>10.51247241194734</v>
+        <v>10.51247246019061</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>1.787894507393719</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.0464932614013949</v>
+        <v>0.0464932613910926</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>49.89878723566674</v>
+        <v>49.89878730562882</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>29.50973018677561</v>
+        <v>29.50973019397893</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.1892592263872863</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.0291312052080315</v>
+        <v>0.0291312052389402</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>46.28129598856892</v>
+        <v>46.2812960131929</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>12.93819738776076</v>
+        <v>12.93819722589178</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.8358651483913635</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.0415195026323594</v>
+        <v>-0.0415195026117587</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>45.40923636903661</v>
+        <v>45.4092363990372</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>15.9994025866516</v>
+        <v>15.9994026000481</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.3345619315422479</v>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>344.6205923617439</v>
+        <v>344.6205923617438</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>69.7</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>41.51972472922288</v>
+        <v>41.51972473181976</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>17.27755574034018</v>
+        <v>17.27755573500607</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.4388308517117974</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.4208327070214537</v>
+        <v>0.4208327071244833</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4318,7 +4318,7 @@
         <v>45.311548594078</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>21.17974308230895</v>
+        <v>21.1797430643264</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.0258545151225515</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.0017758928077551</v>
+        <v>0.0017758927871598</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>52.94284093054748</v>
+        <v>52.94284092517208</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>8.391078854134728</v>
+        <v>8.391078879284182</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.5176056641686142</v>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>49.22656191718546</v>
+        <v>49.22656237582801</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>11.16743397721342</v>
+        <v>11.16743399310105</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.9258614980445508</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.0407918424859618</v>
+        <v>0.040791842503621</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>48.51220901062901</v>
+        <v>48.51220891310973</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>13.07883764282984</v>
+        <v>13.07883754643277</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.2668226654170578</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.4559629286643467</v>
+        <v>-0.4559629283140562</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,7 +4527,7 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>54.43748636460417</v>
+        <v>54.43748638967728</v>
       </c>
       <c r="I77" s="2" t="n">
         <v>22.19787643486348</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.4999337155178392</v>
+        <v>0.4999337154560176</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>326.7347828857845</v>
+        <v>326.7347828857846</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>412</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>45.15748999570672</v>
+        <v>45.15749001467479</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>8.165077412666923</v>
+        <v>8.165077429541601</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.2402832464634738</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-1.136527824415174</v>
+        <v>-1.136527824621186</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>322.3023664125197</v>
+        <v>322.302366412524</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>51</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>43.1919690206711</v>
+        <v>43.19196893741344</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>9.444724956286535</v>
+        <v>9.444725035095598</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>1.246051462242154</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.0266107558188365</v>
+        <v>-0.0266107557776273</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>37.70268301805562</v>
+        <v>37.70268303386835</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>19.91332230406956</v>
+        <v>19.91332229994196</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.3363047400516636</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-17.23431402616788</v>
+        <v>-17.2343140257558</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4725,7 +4725,7 @@
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>319.4928674430854</v>
+        <v>319.4928674430853</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>1530</v>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>46.36378420449738</v>
+        <v>46.3637842240508</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>14.53493402150338</v>
+        <v>14.53493405065067</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.335084557587092</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-23.03758894280538</v>
+        <v>-23.03758894672034</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>55.05746522428631</v>
+        <v>55.0574647690319</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>15.63255877127347</v>
+        <v>15.63255880519765</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.7633969650774827</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.0125232581045694</v>
+        <v>-0.0125232577130676</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>47.24901167068825</v>
+        <v>47.24901165534814</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>9.331955158453816</v>
+        <v>9.33195505922318</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.1999522804176186</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.1516932618139457</v>
+        <v>0.1516932618448554</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>42.92351265023769</v>
+        <v>42.92351270016616</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>29.63784018824169</v>
+        <v>29.6378401882417</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.3033643822283974</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.3388584251234423</v>
+        <v>-0.3388584251955637</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,7 +4951,7 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>47.33372237938669</v>
+        <v>47.33372239767546</v>
       </c>
       <c r="I85" s="2" t="n">
         <v>17.10191097450986</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.0036963860596314</v>
+        <v>-0.0036963859566039</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>288.4548226217462</v>
+        <v>288.454822621746</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>82.3</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>45.75095614132883</v>
+        <v>45.75095641830281</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>13.94461242522091</v>
+        <v>13.94461235866969</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.6403460571916633</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.2965934580430136</v>
+        <v>0.2965934572187685</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>50.49085098261284</v>
+        <v>50.49085074411749</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>12.55513202160818</v>
+        <v>12.55513224158592</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>1.62343459484132</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.1213603339883574</v>
+        <v>0.1213603345035025</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5096,7 +5096,7 @@
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>283.8633905955883</v>
+        <v>283.8633905955882</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>209.5</v>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>41.62341350278633</v>
+        <v>41.6234135494498</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>12.15538149636485</v>
+        <v>12.15538151427203</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.332508490117131</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.0108765455555888</v>
+        <v>-0.0108765461737343</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>280.3097969186821</v>
+        <v>280.3097969186824</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>96.8</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>46.09711529734605</v>
+        <v>46.09711559661935</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>10.92089896110866</v>
+        <v>10.92089896110865</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.641946204768259</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.0199639995715463</v>
+        <v>0.0199639993654718</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>279.722283575741</v>
+        <v>279.7222835757408</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>113</v>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>53.77027259367529</v>
+        <v>53.77027263640132</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>13.87008615017612</v>
+        <v>13.87008616059449</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.6258834396525222</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.4863430399059389</v>
+        <v>0.4863430402150366</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>41.60083965360595</v>
+        <v>41.60083912676578</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>17.57008105511164</v>
+        <v>17.57008104591565</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.7003234123180839</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.1415884160124819</v>
+        <v>-0.1415884158682428</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5322,7 +5322,7 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>48.46548197816509</v>
+        <v>48.46548197560504</v>
       </c>
       <c r="I92" s="2" t="n">
         <v>9.678042294048854</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>3.29630889517877</v>
+        <v>3.296308895384819</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>38.90267581408174</v>
+        <v>38.90267472591915</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>25.0670743646054</v>
+        <v>25.06707505837024</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.5733843133584536</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.0360409965195589</v>
+        <v>0.0360409968286455</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5414,7 +5414,7 @@
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>260.4610578039624</v>
+        <v>260.4610578039632</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>41.4</v>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>49.91367464634831</v>
+        <v>49.91367467182027</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>11.00547870468412</v>
+        <v>11.00547871075513</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>1.2360394854377</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.1973740399775023</v>
+        <v>0.1973740399671954</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>37.79188060992104</v>
+        <v>37.79188046827763</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>26.03791619167086</v>
+        <v>26.03791649979354</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.5826557882460266</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.1685064753163809</v>
+        <v>0.1685064757284906</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>241.7573065478441</v>
+        <v>241.7573065478444</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>110.5</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>38.96565003426014</v>
+        <v>38.96565007686494</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>27.41533882070444</v>
+        <v>27.41533883992354</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.4247648389105568</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.1428655266598013</v>
+        <v>-0.1428655265773857</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>239.0563385192111</v>
+        <v>239.0563385192113</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>25.25</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>40.34641565356581</v>
+        <v>40.34641585446634</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>10.5649980482419</v>
+        <v>10.56499804530666</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.3521453903540544</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.0611514874421841</v>
+        <v>0.061151487545212</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5626,7 +5626,7 @@
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>238.3441852836849</v>
+        <v>238.3441852836837</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>5415</v>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>47.3425138522506</v>
+        <v>47.34251386254056</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>12.0016963799206</v>
+        <v>12.00169647970462</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.5303222279471514</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>14.58219559201653</v>
+        <v>14.58219558459895</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>39.89543620445682</v>
+        <v>39.89543650246283</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>15.17051908727227</v>
+        <v>15.17051919777138</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.6861138362604273</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.0039333712672736</v>
+        <v>-0.0039333715145379</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,7 +5746,7 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>44.30780707882468</v>
+        <v>44.3078070545006</v>
       </c>
       <c r="I100" s="2" t="n">
         <v>36.43845471916114</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.1371158929345433</v>
+        <v>0.1371158929551469</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>217.8255547095977</v>
+        <v>217.8255547095976</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>879</v>
@@ -5802,7 +5802,7 @@
         <v>37.98699343872535</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>18.80190184560387</v>
+        <v>18.80190181495975</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.6084751477765469</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-1.979010483689155</v>
+        <v>-1.979010480598255</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>34.42493330510166</v>
+        <v>34.42493297874039</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>13.30479039063131</v>
+        <v>13.30479054484671</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.514791135031893</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.0520320577022783</v>
+        <v>0.0520320581966828</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>208.9388482070138</v>
+        <v>208.9388482070135</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>42.85</v>
@@ -5908,7 +5908,7 @@
         <v>42.02876394873476</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>17.00784704889255</v>
+        <v>17.00784705078256</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.5752956218348082</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.1880660907081617</v>
+        <v>0.188066090811181</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>40.58252876442935</v>
+        <v>40.58252879748964</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>15.19398287885846</v>
+        <v>15.19398285918395</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.283038536190505</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.2108127003754232</v>
+        <v>0.2108127003548148</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>47.59814510762627</v>
+        <v>47.59814513697284</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>9.79183020897079</v>
+        <v>9.791830131972061</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.2029733890584552</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.454031267487917</v>
+        <v>-0.4540312674055128</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>41.12935780239491</v>
+        <v>41.12935781247861</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>21.7592091179905</v>
+        <v>21.7592091181699</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.2721286845972557</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.0308807551060936</v>
+        <v>0.0308807550957894</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6120,7 +6120,7 @@
         <v>32.64488462725652</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>44.79973580647071</v>
+        <v>44.79973590516246</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.2236491775487307</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.0402282386728288</v>
+        <v>0.0402282387243438</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>42.57860504141423</v>
+        <v>42.57860506298858</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>7.104446560858931</v>
+        <v>7.104446458269309</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.406630448438915</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.0911280502261935</v>
+        <v>-0.0911280501643818</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>179.6655489594881</v>
+        <v>179.6655489594883</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>18.4</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>46.75410530755013</v>
+        <v>46.75410528746463</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>4.383104840893759</v>
+        <v>4.383104756524665</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.3316587358170433</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.136282754270298</v>
+        <v>-0.1362827542187847</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>51.54621104753953</v>
+        <v>51.54621129015008</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>11.73818705462402</v>
+        <v>11.73818704586337</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.5492099394842883</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.2014240423626525</v>
+        <v>0.2014240415384234</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>155.804205017652</v>
+        <v>155.8042050176516</v>
       </c>
       <c r="E111" s="2" t="n">
         <v>49.15</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>47.12795400677779</v>
+        <v>47.12795405626611</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>10.8383568755214</v>
+        <v>10.83835688232522</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.4022046388043475</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.0637214177042897</v>
+        <v>0.0637214176836836</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>46.81199547501882</v>
+        <v>46.81199567266594</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>8.653018608308923</v>
+        <v>8.653018608308919</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.3360373873426625</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.1512677818147805</v>
+        <v>0.1512677816499303</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>50.63805034766321</v>
+        <v>50.63805050570424</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>18.01217968197022</v>
+        <v>18.01217964802071</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.515510380048391</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.0794412769759196</v>
+        <v>-0.0794412773290734</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>42.06665102820589</v>
+        <v>42.06665130275145</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>7.749668534210134</v>
+        <v>7.749668470582674</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.4309727197575089</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.1108212976098693</v>
+        <v>0.1108212976922873</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>83.9963318467918</v>
+        <v>83.99633184679178</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>19.65</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>46.72785904238908</v>
+        <v>46.72785902654893</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>15.56384328870683</v>
+        <v>15.56384340969484</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>1.242251007067564</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.0022391157767619</v>
+        <v>-0.002239115653127</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>

</xml_diff>